<commit_message>
fix(grouping): reconcile กลุ่มย่อย Metier ใน Excel ให้ตรง SKILL §3 (100%)
ก่อนหน้านี้กลุ่มย่อย Metier บางตัวไม่อยู่ในรายการที่ SKILL นิยาม (drift) — แก้ 29 โครงการ:
- Software: System Development → Smart City/Platform Development (+ Mobile/Server-IT
  สำหรับเคสมือถือ/ซ่อมคอมพ์) · Cybersecurity/Certificate + Software/License → Server/IT Infrastructure
- Creative: แยก "Content Creation / Graphic Design" → Content Creation + Graphic Design
- Marketing → 0 (ตาม SKILL "อย่าฝืน promote"): ย้าย Brand/Corporate Image → Media/Public Relations

- scripts/conform_to_skill.py: migration แก้ col กลุ่มหลัก/กลุ่มย่อย + regenerate ชีตสรุปกลุ่ม
- reclassify.py: METIER_RULES ใช้ชื่อ SKILL §3 ทั้งหมด → audit metierSubGroup 96.1%
- ผล: กลุ่มย่อย Metier ตรง SKILL §3 ครบ 100% (Software 3 · Creative 4 · Media 2 · Marketing 0)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/โครงสร้างโฟลเดอร์_รวม_TOR.xlsx
+++ b/โครงสร้างโฟลเดอร์_รวม_TOR.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17400" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="แผนผังโฟลเดอร์" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="พจนานุกรมข้อมูล" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ภาพรวม" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="รายการโครงการทั้งหมด" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="สรุปกลุ่ม" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="เช็คการอ่านไฟล์" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOR" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="แผนผังโฟลเดอร์" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="พจนานุกรมข้อมูล" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ภาพรวม" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="รายการโครงการทั้งหมด" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="สรุปกลุ่ม" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="เช็คการอ่านไฟล์" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="TOR" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'รายการโครงการทั้งหมด'!$A$1:$H$311</definedName>
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -166,8 +166,11 @@
       <color rgb="FF808000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -217,6 +220,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF6CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -291,7 +299,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -372,6 +380,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1388,11 +1398,11 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A10:E10"/>
-    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B34:E34"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B37:E37"/>
     <mergeCell ref="A27:E27"/>
     <mergeCell ref="B32:E32"/>
   </mergeCells>
@@ -4500,7 +4510,7 @@
       </c>
       <c r="H64" s="24" t="inlineStr">
         <is>
-          <t>Software/License</t>
+          <t>Server/IT Infrastructure</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4928,7 @@
       </c>
       <c r="H75" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -6704,7 +6714,7 @@
       </c>
       <c r="H122" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -6780,7 +6790,7 @@
       </c>
       <c r="H124" s="24" t="inlineStr">
         <is>
-          <t>Content Creation / Graphic Design</t>
+          <t>Graphic Design</t>
         </is>
       </c>
     </row>
@@ -6818,7 +6828,7 @@
       </c>
       <c r="H125" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -6927,12 +6937,12 @@
       </c>
       <c r="G128" s="25" t="inlineStr">
         <is>
-          <t>Marketing Metier</t>
+          <t>Media Metier</t>
         </is>
       </c>
       <c r="H128" s="24" t="inlineStr">
         <is>
-          <t>Brand/Corporate Image</t>
+          <t>Public Relations</t>
         </is>
       </c>
     </row>
@@ -7198,7 +7208,7 @@
       </c>
       <c r="H135" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -7844,7 +7854,7 @@
       </c>
       <c r="H152" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -8186,7 +8196,7 @@
       </c>
       <c r="H161" s="24" t="inlineStr">
         <is>
-          <t>Cybersecurity/Certificate</t>
+          <t>Server/IT Infrastructure</t>
         </is>
       </c>
     </row>
@@ -8262,7 +8272,7 @@
       </c>
       <c r="H163" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -8832,7 +8842,7 @@
       </c>
       <c r="H178" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -9364,7 +9374,7 @@
       </c>
       <c r="H192" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -9820,7 +9830,7 @@
       </c>
       <c r="H204" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -9934,7 +9944,7 @@
       </c>
       <c r="H207" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -10238,7 +10248,7 @@
       </c>
       <c r="H215" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -10314,7 +10324,7 @@
       </c>
       <c r="H217" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -10428,7 +10438,7 @@
       </c>
       <c r="H220" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Server/IT Infrastructure</t>
         </is>
       </c>
     </row>
@@ -10504,7 +10514,7 @@
       </c>
       <c r="H222" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -10694,7 +10704,7 @@
       </c>
       <c r="H227" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Mobile Application</t>
         </is>
       </c>
     </row>
@@ -11226,7 +11236,7 @@
       </c>
       <c r="H241" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -11416,7 +11426,7 @@
       </c>
       <c r="H246" s="24" t="inlineStr">
         <is>
-          <t>Cybersecurity/Certificate</t>
+          <t>Server/IT Infrastructure</t>
         </is>
       </c>
     </row>
@@ -11454,7 +11464,7 @@
       </c>
       <c r="H247" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -11720,7 +11730,7 @@
       </c>
       <c r="H254" s="24" t="inlineStr">
         <is>
-          <t>Cybersecurity/Certificate</t>
+          <t>Server/IT Infrastructure</t>
         </is>
       </c>
     </row>
@@ -11834,7 +11844,7 @@
       </c>
       <c r="H257" s="24" t="inlineStr">
         <is>
-          <t>Content Creation / Graphic Design</t>
+          <t>Content Creation</t>
         </is>
       </c>
     </row>
@@ -12328,7 +12338,7 @@
       </c>
       <c r="H270" s="24" t="inlineStr">
         <is>
-          <t>Content Creation / Graphic Design</t>
+          <t>Content Creation</t>
         </is>
       </c>
     </row>
@@ -12552,7 +12562,7 @@
       </c>
       <c r="H276" s="24" t="inlineStr">
         <is>
-          <t>Content Creation / Graphic Design</t>
+          <t>Content Creation</t>
         </is>
       </c>
     </row>
@@ -12662,7 +12672,7 @@
       </c>
       <c r="H279" s="24" t="inlineStr">
         <is>
-          <t>Content Creation / Graphic Design</t>
+          <t>Content Creation</t>
         </is>
       </c>
     </row>
@@ -13270,7 +13280,7 @@
       </c>
       <c r="H295" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -13726,7 +13736,7 @@
       </c>
       <c r="H307" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Smart City/Platform Development</t>
         </is>
       </c>
     </row>
@@ -13894,1073 +13904,764 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D70"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:C67"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="39" min="1" max="1"/>
-    <col width="42" customWidth="1" style="39" min="2" max="2"/>
-    <col width="16" customWidth="1" style="39" min="3" max="3"/>
-    <col width="34" customWidth="1" style="39" min="4" max="4"/>
+    <col width="26" customWidth="1" style="39" min="1" max="1"/>
+    <col width="38" customWidth="1" style="39" min="2" max="2"/>
+    <col width="14" customWidth="1" style="39" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" customHeight="1" s="39">
-      <c r="A1" s="43" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="48" t="inlineStr">
         <is>
           <t>สรุปการจัดกลุ่ม (ชุดเดียว) : กลุ่มหลัก → กลุ่มย่อย</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="45" t="inlineStr">
-        <is>
-          <t>กลุ่มหลักรวม 7 หมวดงาน + Software/Creative/Media/Marketing Metier (โครงการที่เป็นโอกาส Metier ยึดกลุ่ม Metier ก่อน · แถว Metier ไฮไลต์เหลือง)</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>กลุ่มหลักรวม 7 หมวดงาน + Software/Creative/Media/Marketing Metier (กลุ่มย่อย Metier ตรงตาม SKILL thai-municipal-project-grouping §3)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>กลุ่มหลัก</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="48" t="inlineStr">
         <is>
           <t>กลุ่มย่อย</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="48" t="inlineStr">
         <is>
           <t>จำนวนโครงการ</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>ขอบเขต skill.md</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="37" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>1. บริหารจัดการ</t>
         </is>
       </c>
-      <c r="B5" s="37" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>บำรุงรักษา/ซ่อม</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
+      <c r="C5" t="n">
         <v>23</v>
       </c>
-      <c r="D5" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="37" t="n"/>
-      <c r="B6" s="37" t="inlineStr">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
         <is>
           <t>เช่า-จ้างเหมาบริการ (ทั่วไป)</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" t="n">
         <v>7</v>
       </c>
-      <c r="D6" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" s="37" t="n"/>
-      <c r="B7" s="37" t="inlineStr">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
         <is>
           <t>รักษาความปลอดภัย</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
     </row>
     <row r="8">
-      <c r="A8" s="37" t="n"/>
-      <c r="B8" s="37" t="inlineStr">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
         <is>
           <t>ระบบสารสนเทศ/ดิจิทัล/ซอฟต์แวร์</t>
         </is>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" s="37" t="n"/>
-      <c r="B9" s="37" t="inlineStr">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
         <is>
           <t>ป้องกันสาธารณภัย-ดับเพลิง</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
     </row>
     <row r="10">
-      <c r="A10" s="37" t="n"/>
-      <c r="B10" s="37" t="inlineStr">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
         <is>
           <t>เครือข่าย/อินเทอร์เน็ต/IT บริการ</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="37" t="n"/>
-      <c r="B11" s="37" t="inlineStr">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>จัดหาเครื่องแต่งกาย/วัสดุทั่วไป</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
         <is>
           <t>ฝึกอบรม-พัฒนาบุคลากร</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C12" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="37" t="n"/>
-      <c r="B12" s="37" t="inlineStr">
-        <is>
-          <t>จัดหาเครื่องแต่งกาย/วัสดุทั่วไป</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="n">
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>งานติดตั้ง/บริการอื่น</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ตรวจสอบ-ที่ปรึกษา</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>บริการสอบเทียบ/วิชาการ</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="48" t="inlineStr">
+        <is>
+          <t>รวม 1. บริหารจัดการ</t>
+        </is>
+      </c>
+      <c r="B16" s="48" t="inlineStr"/>
+      <c r="C16" s="48" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2. โครงสร้างพื้นฐาน</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>อาคาร/สิ่งก่อสร้าง/ลาน</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ประปา-แหล่งน้ำ</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ไฟฟ้า-แสงสว่าง/สาธารณูปโภค</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ถนน-คอนกรีต (คสล.)</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ถนน-แอสฟัลท์/ลาดยาง</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ถนน-บำรุง/ทั่วไป</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ระบบระบายน้ำ/ป้องกันตลิ่ง</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>งานระบบประกอบอาคาร (ปรับ/ระบายอากาศ)</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>วัสดุก่อสร้าง</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ไฟฟ้า-พลังงานแสงอาทิตย์</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>สะพาน/ทางเชื่อม</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="48" t="inlineStr">
+        <is>
+          <t>รวม 2. โครงสร้างพื้นฐาน</t>
+        </is>
+      </c>
+      <c r="B28" s="48" t="inlineStr"/>
+      <c r="C28" s="48" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>3. คุณภาพชีวิต</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>บริการตรวจวินิจฉัย/แล็บ</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>เวชภัณฑ์ยา/วัสดุการแพทย์</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>บริการสาธารณสุข</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>สวัสดิการ-ช่วยเหลือสังคม</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="48" t="inlineStr">
+        <is>
+          <t>รวม 3. คุณภาพชีวิต</t>
+        </is>
+      </c>
+      <c r="B33" s="48" t="inlineStr"/>
+      <c r="C33" s="48" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>4. ชุมชนเข้มแข็ง</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ชุมชน-ท่องเที่ยว-พลังงานชุมชน</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="48" t="inlineStr">
+        <is>
+          <t>รวม 4. ชุมชนเข้มแข็ง</t>
+        </is>
+      </c>
+      <c r="B35" s="48" t="inlineStr"/>
+      <c r="C35" s="48" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>5. การศึกษา ศาสนา กีฬา</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>สื่อ/อุปกรณ์การเรียนการสอน</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>สนามกีฬา</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="37" t="n"/>
-      <c r="B13" s="37" t="inlineStr">
-        <is>
-          <t>บริการสอบเทียบ/วิชาการ</t>
-        </is>
-      </c>
-      <c r="C13" s="14" t="n">
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>กีฬา-การแข่งขัน</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="37" t="n"/>
-      <c r="B14" s="37" t="inlineStr">
-        <is>
-          <t>งานติดตั้ง/บริการอื่น</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="n">
+    </row>
+    <row r="39">
+      <c r="A39" s="48" t="inlineStr">
+        <is>
+          <t>รวม 5. การศึกษา ศาสนา กีฬา</t>
+        </is>
+      </c>
+      <c r="B39" s="48" t="inlineStr"/>
+      <c r="C39" s="48" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>6. ความสะอาดและสิ่งแวดล้อม</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>กำจัดขยะ/ของเสีย</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ทำความสะอาด</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="48" t="inlineStr">
+        <is>
+          <t>รวม 6. ความสะอาดและสิ่งแวดล้อม</t>
+        </is>
+      </c>
+      <c r="B42" s="48" t="inlineStr"/>
+      <c r="C42" s="48" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>7. ครุภัณฑ์</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-วิทยาศาสตร์/การแพทย์</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-ยานพาหนะ</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์/วัสดุ-ดาราศาสตร์-วิจัย</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-คอมพิวเตอร์/IT</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-สำนักงาน</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-ก่อสร้าง/เครื่องจักร</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-โฆษณา/Display/CCTV</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-ไฟฟ้าและวิทยุ</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="37" t="n"/>
-      <c r="B15" s="37" t="inlineStr">
-        <is>
-          <t>ตรวจสอบ-ที่ปรึกษา</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="n">
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์/วัสดุ-โซลาร์</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>รวม 1. บริหารจัดการ</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="n"/>
-      <c r="C16" s="17" t="n">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="37" t="inlineStr">
-        <is>
-          <t>2. โครงสร้างพื้นฐาน</t>
-        </is>
-      </c>
-      <c r="B17" s="37" t="inlineStr">
-        <is>
-          <t>อาคาร/สิ่งก่อสร้าง/ลาน</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="n">
+    </row>
+    <row r="52">
+      <c r="A52" s="48" t="inlineStr">
+        <is>
+          <t>รวม 7. ครุภัณฑ์</t>
+        </is>
+      </c>
+      <c r="B52" s="48" t="inlineStr"/>
+      <c r="C52" s="48" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="49" t="inlineStr">
+        <is>
+          <t>Software Metier</t>
+        </is>
+      </c>
+      <c r="B53" s="49" t="inlineStr">
+        <is>
+          <t>Smart City/Platform Development</t>
+        </is>
+      </c>
+      <c r="C53" s="49" t="n">
         <v>21</v>
       </c>
-      <c r="D17" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="37" t="n"/>
-      <c r="B18" s="37" t="inlineStr">
-        <is>
-          <t>ประปา-แหล่งน้ำ</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="D18" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="37" t="n"/>
-      <c r="B19" s="37" t="inlineStr">
-        <is>
-          <t>ไฟฟ้า-แสงสว่าง/สาธารณูปโภค</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="n">
-        <v>11</v>
-      </c>
-      <c r="D19" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="37" t="n"/>
-      <c r="B20" s="37" t="inlineStr">
-        <is>
-          <t>ถนน-คอนกรีต (คสล.)</t>
-        </is>
-      </c>
-      <c r="C20" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="D20" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="37" t="n"/>
-      <c r="B21" s="37" t="inlineStr">
-        <is>
-          <t>ถนน-แอสฟัลท์/ลาดยาง</t>
-        </is>
-      </c>
-      <c r="C21" s="14" t="n">
+    </row>
+    <row r="54">
+      <c r="A54" s="49" t="inlineStr"/>
+      <c r="B54" s="49" t="inlineStr">
+        <is>
+          <t>Server/IT Infrastructure</t>
+        </is>
+      </c>
+      <c r="C54" s="49" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="49" t="inlineStr"/>
+      <c r="B55" s="49" t="inlineStr">
+        <is>
+          <t>Mobile Application</t>
+        </is>
+      </c>
+      <c r="C55" s="49" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="48" t="inlineStr">
+        <is>
+          <t>รวม Software Metier</t>
+        </is>
+      </c>
+      <c r="B56" s="48" t="inlineStr"/>
+      <c r="C56" s="48" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="49" t="inlineStr">
+        <is>
+          <t>Creative Metier</t>
+        </is>
+      </c>
+      <c r="B57" s="49" t="inlineStr">
+        <is>
+          <t>Event Marketing/Festival</t>
+        </is>
+      </c>
+      <c r="C57" s="49" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="49" t="inlineStr"/>
+      <c r="B58" s="49" t="inlineStr">
+        <is>
+          <t>Content Creation</t>
+        </is>
+      </c>
+      <c r="C58" s="49" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="49" t="inlineStr"/>
+      <c r="B59" s="49" t="inlineStr">
+        <is>
+          <t>Branding &amp; Display Production</t>
+        </is>
+      </c>
+      <c r="C59" s="49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="49" t="inlineStr"/>
+      <c r="B60" s="49" t="inlineStr">
+        <is>
+          <t>Graphic Design</t>
+        </is>
+      </c>
+      <c r="C60" s="49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="48" t="inlineStr">
+        <is>
+          <t>รวม Creative Metier</t>
+        </is>
+      </c>
+      <c r="B61" s="48" t="inlineStr"/>
+      <c r="C61" s="48" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="49" t="inlineStr">
+        <is>
+          <t>Media Metier</t>
+        </is>
+      </c>
+      <c r="B62" s="49" t="inlineStr">
+        <is>
+          <t>Public Relations</t>
+        </is>
+      </c>
+      <c r="C62" s="49" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="49" t="inlineStr"/>
+      <c r="B63" s="49" t="inlineStr">
+        <is>
+          <t>Offline Media</t>
+        </is>
+      </c>
+      <c r="C63" s="49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="48" t="inlineStr">
+        <is>
+          <t>รวม Media Metier</t>
+        </is>
+      </c>
+      <c r="B64" s="48" t="inlineStr"/>
+      <c r="C64" s="48" t="n">
         <v>6</v>
       </c>
-      <c r="D21" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="37" t="n"/>
-      <c r="B22" s="37" t="inlineStr">
-        <is>
-          <t>ระบบระบายน้ำ/ป้องกันตลิ่ง</t>
-        </is>
-      </c>
-      <c r="C22" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D22" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="37" t="n"/>
-      <c r="B23" s="37" t="inlineStr">
-        <is>
-          <t>ถนน-บำรุง/ทั่วไป</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D23" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="37" t="n"/>
-      <c r="B24" s="37" t="inlineStr">
-        <is>
-          <t>วัสดุก่อสร้าง</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="D24" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="37" t="n"/>
-      <c r="B25" s="37" t="inlineStr">
-        <is>
-          <t>งานระบบประกอบอาคาร (ปรับ/ระบายอากาศ)</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="D25" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="37" t="n"/>
-      <c r="B26" s="37" t="inlineStr">
-        <is>
-          <t>ไฟฟ้า-พลังงานแสงอาทิตย์</t>
-        </is>
-      </c>
-      <c r="C26" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="D26" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="37" t="n"/>
-      <c r="B27" s="37" t="inlineStr">
-        <is>
-          <t>สะพาน/ทางเชื่อม</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>รวม 2. โครงสร้างพื้นฐาน</t>
-        </is>
-      </c>
-      <c r="B28" s="16" t="n"/>
-      <c r="C28" s="17" t="n">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="37" t="inlineStr">
-        <is>
-          <t>3. คุณภาพชีวิต</t>
-        </is>
-      </c>
-      <c r="B29" s="37" t="inlineStr">
-        <is>
-          <t>บริการตรวจวินิจฉัย/แล็บ</t>
-        </is>
-      </c>
-      <c r="C29" s="14" t="n">
-        <v>16</v>
-      </c>
-      <c r="D29" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="37" t="n"/>
-      <c r="B30" s="37" t="inlineStr">
-        <is>
-          <t>เวชภัณฑ์ยา/วัสดุการแพทย์</t>
-        </is>
-      </c>
-      <c r="C30" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="D30" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="37" t="n"/>
-      <c r="B31" s="37" t="inlineStr">
-        <is>
-          <t>บริการสาธารณสุข</t>
-        </is>
-      </c>
-      <c r="C31" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="D31" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="37" t="n"/>
-      <c r="B32" s="37" t="inlineStr">
-        <is>
-          <t>สวัสดิการ-ช่วยเหลือสังคม</t>
-        </is>
-      </c>
-      <c r="C32" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
-        <is>
-          <t>รวม 3. คุณภาพชีวิต</t>
-        </is>
-      </c>
-      <c r="B33" s="16" t="n"/>
-      <c r="C33" s="17" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="37" t="inlineStr">
-        <is>
-          <t>4. ชุมชนเข้มแข็ง</t>
-        </is>
-      </c>
-      <c r="B34" s="37" t="inlineStr">
-        <is>
-          <t>ชุมชน-ท่องเที่ยว-พลังงานชุมชน</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D34" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="15" t="inlineStr">
-        <is>
-          <t>รวม 4. ชุมชนเข้มแข็ง</t>
-        </is>
-      </c>
-      <c r="B35" s="16" t="n"/>
-      <c r="C35" s="17" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="37" t="inlineStr">
-        <is>
-          <t>5. การศึกษา ศาสนา กีฬา</t>
-        </is>
-      </c>
-      <c r="B36" s="37" t="inlineStr">
-        <is>
-          <t>สื่อ/อุปกรณ์การเรียนการสอน</t>
-        </is>
-      </c>
-      <c r="C36" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D36" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="37" t="n"/>
-      <c r="B37" s="37" t="inlineStr">
-        <is>
-          <t>สนามกีฬา</t>
-        </is>
-      </c>
-      <c r="C37" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D37" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="37" t="n"/>
-      <c r="B38" s="37" t="inlineStr">
-        <is>
-          <t>กีฬา-การแข่งขัน</t>
-        </is>
-      </c>
-      <c r="C38" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="15" t="inlineStr">
-        <is>
-          <t>รวม 5. การศึกษา ศาสนา กีฬา</t>
-        </is>
-      </c>
-      <c r="B39" s="16" t="n"/>
-      <c r="C39" s="17" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="37" t="inlineStr">
-        <is>
-          <t>6. ความสะอาดและสิ่งแวดล้อม</t>
-        </is>
-      </c>
-      <c r="B40" s="37" t="inlineStr">
-        <is>
-          <t>กำจัดขยะ/ของเสีย</t>
-        </is>
-      </c>
-      <c r="C40" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="D40" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="37" t="n"/>
-      <c r="B41" s="37" t="inlineStr">
-        <is>
-          <t>ทำความสะอาด</t>
-        </is>
-      </c>
-      <c r="C41" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="D41" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="15" t="inlineStr">
-        <is>
-          <t>รวม 6. ความสะอาดและสิ่งแวดล้อม</t>
-        </is>
-      </c>
-      <c r="B42" s="16" t="n"/>
-      <c r="C42" s="17" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="37" t="inlineStr">
-        <is>
-          <t>7. ครุภัณฑ์</t>
-        </is>
-      </c>
-      <c r="B43" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-วิทยาศาสตร์/การแพทย์</t>
-        </is>
-      </c>
-      <c r="C43" s="14" t="n">
-        <v>20</v>
-      </c>
-      <c r="D43" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="37" t="n"/>
-      <c r="B44" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-ยานพาหนะ</t>
-        </is>
-      </c>
-      <c r="C44" s="14" t="n">
-        <v>18</v>
-      </c>
-      <c r="D44" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="37" t="n"/>
-      <c r="B45" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์/วัสดุ-ดาราศาสตร์-วิจัย</t>
-        </is>
-      </c>
-      <c r="C45" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="D45" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="37" t="n"/>
-      <c r="B46" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-คอมพิวเตอร์/IT</t>
-        </is>
-      </c>
-      <c r="C46" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="D46" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="37" t="n"/>
-      <c r="B47" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-สำนักงาน</t>
-        </is>
-      </c>
-      <c r="C47" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D47" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="37" t="n"/>
-      <c r="B48" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-ก่อสร้าง/เครื่องจักร</t>
-        </is>
-      </c>
-      <c r="C48" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D48" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="37" t="n"/>
-      <c r="B49" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-โฆษณา/Display/CCTV</t>
-        </is>
-      </c>
-      <c r="C49" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D49" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="37" t="n"/>
-      <c r="B50" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-ไฟฟ้าและวิทยุ</t>
-        </is>
-      </c>
-      <c r="C50" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="37" t="n"/>
-      <c r="B51" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์/วัสดุ-โซลาร์</t>
-        </is>
-      </c>
-      <c r="C51" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="15" t="inlineStr">
-        <is>
-          <t>รวม 7. ครุภัณฑ์</t>
-        </is>
-      </c>
-      <c r="B52" s="16" t="n"/>
-      <c r="C52" s="17" t="n">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="26" t="inlineStr">
-        <is>
-          <t>Software Metier</t>
-        </is>
-      </c>
-      <c r="B53" s="37" t="inlineStr">
-        <is>
-          <t>System Development</t>
-        </is>
-      </c>
-      <c r="C53" s="14" t="n">
-        <v>19</v>
-      </c>
-      <c r="D53" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="37" t="n"/>
-      <c r="B54" s="37" t="inlineStr">
-        <is>
-          <t>Smart City/Platform Development</t>
-        </is>
-      </c>
-      <c r="C54" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D54" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="37" t="n"/>
-      <c r="B55" s="37" t="inlineStr">
-        <is>
-          <t>Cybersecurity/Certificate</t>
-        </is>
-      </c>
-      <c r="C55" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="D55" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="37" t="n"/>
-      <c r="B56" s="37" t="inlineStr">
-        <is>
-          <t>Software/License</t>
-        </is>
-      </c>
-      <c r="C56" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="37" t="n"/>
-      <c r="B57" s="37" t="inlineStr">
-        <is>
-          <t>Mobile Application</t>
-        </is>
-      </c>
-      <c r="C57" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D57" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="27" t="inlineStr">
-        <is>
-          <t>รวม Software Metier</t>
-        </is>
-      </c>
-      <c r="B58" s="28" t="n"/>
-      <c r="C58" s="29" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="26" t="inlineStr">
-        <is>
-          <t>Creative Metier</t>
-        </is>
-      </c>
-      <c r="B59" s="37" t="inlineStr">
-        <is>
-          <t>Event Marketing/Festival</t>
-        </is>
-      </c>
-      <c r="C59" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="D59" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="37" t="n"/>
-      <c r="B60" s="37" t="inlineStr">
-        <is>
-          <t>Content Creation / Graphic Design</t>
-        </is>
-      </c>
-      <c r="C60" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D60" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="37" t="n"/>
-      <c r="B61" s="37" t="inlineStr">
-        <is>
-          <t>Branding &amp; Display Production</t>
-        </is>
-      </c>
-      <c r="C61" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="27" t="inlineStr">
-        <is>
-          <t>รวม Creative Metier</t>
-        </is>
-      </c>
-      <c r="B62" s="28" t="n"/>
-      <c r="C62" s="29" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="26" t="inlineStr">
-        <is>
-          <t>Media Metier</t>
-        </is>
-      </c>
-      <c r="B63" s="37" t="inlineStr">
-        <is>
-          <t>Public Relations</t>
-        </is>
-      </c>
-      <c r="C63" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D63" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="37" t="n"/>
-      <c r="B64" s="37" t="inlineStr">
-        <is>
-          <t>Offline Media</t>
-        </is>
-      </c>
-      <c r="C64" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
     </row>
     <row r="65">
-      <c r="A65" s="27" t="inlineStr">
-        <is>
-          <t>รวม Media Metier</t>
-        </is>
-      </c>
-      <c r="B65" s="28" t="n"/>
-      <c r="C65" s="29" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="26" t="inlineStr">
-        <is>
-          <t>Marketing Metier</t>
-        </is>
-      </c>
-      <c r="B66" s="37" t="inlineStr">
-        <is>
-          <t>Brand/Corporate Image</t>
-        </is>
-      </c>
-      <c r="C66" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
+      <c r="A65" s="48" t="inlineStr">
+        <is>
+          <t>รวมทั้งหมด</t>
+        </is>
+      </c>
+      <c r="B65" s="48" t="inlineStr"/>
+      <c r="C65" s="48" t="n">
+        <v>310</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="27" t="inlineStr">
-        <is>
-          <t>รวม Marketing Metier</t>
-        </is>
-      </c>
-      <c r="B67" s="28" t="n"/>
-      <c r="C67" s="29" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="18" t="inlineStr">
-        <is>
-          <t>รวมทั้งหมด</t>
-        </is>
-      </c>
-      <c r="B68" s="18" t="n"/>
-      <c r="C68" s="1" t="n">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="69"/>
-    <row r="70">
-      <c r="A70" s="44" t="inlineStr">
-        <is>
-          <t>➜ โครงการที่เป็นโอกาส Metier (Software/Creative/Media/Marketing Metier) = 49 จาก 310 โครงการ</t>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>➜ โครงการที่เป็นโอกาส Metier = 49 จาก 310 โครงการ</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A70:C70"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(grouping): เปลี่ยนกลุ่มย่อย Metier เป็น canonical sub-service (dropdown UI)
ตาม taxonomy ทางการของ Metier (4 dropdown) — กลุ่มหลักคง "X Metier", จับกลุ่มย่อย
เข้าช่องใกล้สุดรายตัว (49 โครงการ), ที่ไม่ตรงช่อง → "อื่น ๆ (ยังไม่จัดประเภท)":
- Software: ERP/CRM Systems 20 · Cyber Security 2 · Mobile Application 2 · อื่นๆ 4
- Creative: Event Marketing 10 · Content Creation 3 · Graphic Design 1 · อื่นๆ 1
- Media: Public Relations 4 · Offline Media 1
- Marketing: Brand Strategy 1
- scripts/apply_canonical_subgroups.py (migration), reclassify.py + README ใช้ชุด canonical

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/โครงสร้างโฟลเดอร์_รวม_TOR.xlsx
+++ b/โครงสร้างโฟลเดอร์_รวม_TOR.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17400" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="แผนผังโฟลเดอร์" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="พจนานุกรมข้อมูล" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ภาพรวม" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="รายการโครงการทั้งหมด" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="สรุปกลุ่ม" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="เช็คการอ่านไฟล์" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOR" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="แผนผังโฟลเดอร์" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="พจนานุกรมข้อมูล" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ภาพรวม" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="รายการโครงการทั้งหมด" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="สรุปกลุ่ม" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="เช็คการอ่านไฟล์" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="TOR" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'รายการโครงการทั้งหมด'!$A$1:$H$311</definedName>
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -166,8 +166,11 @@
       <color rgb="FF808000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -217,6 +220,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF6CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -291,7 +299,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -372,6 +380,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1388,11 +1398,11 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A10:E10"/>
-    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B34:E34"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B37:E37"/>
     <mergeCell ref="A27:E27"/>
     <mergeCell ref="B32:E32"/>
   </mergeCells>
@@ -4500,7 +4510,7 @@
       </c>
       <c r="H64" s="24" t="inlineStr">
         <is>
-          <t>Software/License</t>
+          <t>อื่น ๆ (ยังไม่จัดประเภท)</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4928,7 @@
       </c>
       <c r="H75" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -6704,7 +6714,7 @@
       </c>
       <c r="H122" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -6780,7 +6790,7 @@
       </c>
       <c r="H124" s="24" t="inlineStr">
         <is>
-          <t>Content Creation / Graphic Design</t>
+          <t>Graphic Design</t>
         </is>
       </c>
     </row>
@@ -6818,7 +6828,7 @@
       </c>
       <c r="H125" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -6932,7 +6942,7 @@
       </c>
       <c r="H128" s="24" t="inlineStr">
         <is>
-          <t>Brand/Corporate Image</t>
+          <t>Brand Strategy</t>
         </is>
       </c>
     </row>
@@ -7084,7 +7094,7 @@
       </c>
       <c r="H132" s="24" t="inlineStr">
         <is>
-          <t>Branding &amp; Display Production</t>
+          <t>อื่น ๆ (ยังไม่จัดประเภท)</t>
         </is>
       </c>
     </row>
@@ -7198,7 +7208,7 @@
       </c>
       <c r="H135" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -7844,7 +7854,7 @@
       </c>
       <c r="H152" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -8072,7 +8082,7 @@
       </c>
       <c r="H158" s="24" t="inlineStr">
         <is>
-          <t>Smart City/Platform Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -8186,7 +8196,7 @@
       </c>
       <c r="H161" s="24" t="inlineStr">
         <is>
-          <t>Cybersecurity/Certificate</t>
+          <t>Software Quality Assurance &amp; Cyber Security</t>
         </is>
       </c>
     </row>
@@ -8262,7 +8272,7 @@
       </c>
       <c r="H163" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -8452,7 +8462,7 @@
       </c>
       <c r="H168" s="24" t="inlineStr">
         <is>
-          <t>Event Marketing/Festival</t>
+          <t>Event Marketing</t>
         </is>
       </c>
     </row>
@@ -8680,7 +8690,7 @@
       </c>
       <c r="H174" s="24" t="inlineStr">
         <is>
-          <t>Event Marketing/Festival</t>
+          <t>Event Marketing</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8728,7 @@
       </c>
       <c r="H175" s="24" t="inlineStr">
         <is>
-          <t>Smart City/Platform Development</t>
+          <t>อื่น ๆ (ยังไม่จัดประเภท)</t>
         </is>
       </c>
     </row>
@@ -8832,7 +8842,7 @@
       </c>
       <c r="H178" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -9364,7 +9374,7 @@
       </c>
       <c r="H192" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -9820,7 +9830,7 @@
       </c>
       <c r="H204" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -9934,7 +9944,7 @@
       </c>
       <c r="H207" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -10238,7 +10248,7 @@
       </c>
       <c r="H215" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -10314,7 +10324,7 @@
       </c>
       <c r="H217" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -10428,7 +10438,7 @@
       </c>
       <c r="H220" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>อื่น ๆ (ยังไม่จัดประเภท)</t>
         </is>
       </c>
     </row>
@@ -10504,7 +10514,7 @@
       </c>
       <c r="H222" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -10694,7 +10704,7 @@
       </c>
       <c r="H227" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>Mobile Application</t>
         </is>
       </c>
     </row>
@@ -11074,7 +11084,7 @@
       </c>
       <c r="H237" s="24" t="inlineStr">
         <is>
-          <t>Event Marketing/Festival</t>
+          <t>Event Marketing</t>
         </is>
       </c>
     </row>
@@ -11226,7 +11236,7 @@
       </c>
       <c r="H241" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -11416,7 +11426,7 @@
       </c>
       <c r="H246" s="24" t="inlineStr">
         <is>
-          <t>Cybersecurity/Certificate</t>
+          <t>อื่น ๆ (ยังไม่จัดประเภท)</t>
         </is>
       </c>
     </row>
@@ -11454,7 +11464,7 @@
       </c>
       <c r="H247" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -11720,7 +11730,7 @@
       </c>
       <c r="H254" s="24" t="inlineStr">
         <is>
-          <t>Cybersecurity/Certificate</t>
+          <t>Software Quality Assurance &amp; Cyber Security</t>
         </is>
       </c>
     </row>
@@ -11834,7 +11844,7 @@
       </c>
       <c r="H257" s="24" t="inlineStr">
         <is>
-          <t>Content Creation / Graphic Design</t>
+          <t>Content Creation</t>
         </is>
       </c>
     </row>
@@ -12214,7 +12224,7 @@
       </c>
       <c r="H267" s="24" t="inlineStr">
         <is>
-          <t>Event Marketing/Festival</t>
+          <t>Event Marketing</t>
         </is>
       </c>
     </row>
@@ -12328,7 +12338,7 @@
       </c>
       <c r="H270" s="24" t="inlineStr">
         <is>
-          <t>Content Creation / Graphic Design</t>
+          <t>Content Creation</t>
         </is>
       </c>
     </row>
@@ -12552,7 +12562,7 @@
       </c>
       <c r="H276" s="24" t="inlineStr">
         <is>
-          <t>Content Creation / Graphic Design</t>
+          <t>Content Creation</t>
         </is>
       </c>
     </row>
@@ -12590,7 +12600,7 @@
       </c>
       <c r="H277" s="24" t="inlineStr">
         <is>
-          <t>Event Marketing/Festival</t>
+          <t>Event Marketing</t>
         </is>
       </c>
     </row>
@@ -12628,7 +12638,7 @@
       </c>
       <c r="H278" s="24" t="inlineStr">
         <is>
-          <t>Event Marketing/Festival</t>
+          <t>Event Marketing</t>
         </is>
       </c>
     </row>
@@ -12662,7 +12672,7 @@
       </c>
       <c r="H279" s="24" t="inlineStr">
         <is>
-          <t>Content Creation / Graphic Design</t>
+          <t>Event Marketing</t>
         </is>
       </c>
     </row>
@@ -13004,7 +13014,7 @@
       </c>
       <c r="H288" s="24" t="inlineStr">
         <is>
-          <t>Smart City/Platform Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -13042,7 +13052,7 @@
       </c>
       <c r="H289" s="24" t="inlineStr">
         <is>
-          <t>Smart City/Platform Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -13270,7 +13280,7 @@
       </c>
       <c r="H295" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -13346,7 +13356,7 @@
       </c>
       <c r="H297" s="24" t="inlineStr">
         <is>
-          <t>Event Marketing/Festival</t>
+          <t>Event Marketing</t>
         </is>
       </c>
     </row>
@@ -13384,7 +13394,7 @@
       </c>
       <c r="H298" s="24" t="inlineStr">
         <is>
-          <t>Event Marketing/Festival</t>
+          <t>Event Marketing</t>
         </is>
       </c>
     </row>
@@ -13536,7 +13546,7 @@
       </c>
       <c r="H302" s="24" t="inlineStr">
         <is>
-          <t>Event Marketing/Festival</t>
+          <t>Event Marketing</t>
         </is>
       </c>
     </row>
@@ -13726,7 +13736,7 @@
       </c>
       <c r="H307" s="24" t="inlineStr">
         <is>
-          <t>System Development</t>
+          <t>ERP/CRM Systems</t>
         </is>
       </c>
     </row>
@@ -13894,1073 +13904,794 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D70"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:C68"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="39" min="1" max="1"/>
+    <col width="26" customWidth="1" style="39" min="1" max="1"/>
     <col width="42" customWidth="1" style="39" min="2" max="2"/>
-    <col width="16" customWidth="1" style="39" min="3" max="3"/>
-    <col width="34" customWidth="1" style="39" min="4" max="4"/>
+    <col width="14" customWidth="1" style="39" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" customHeight="1" s="39">
-      <c r="A1" s="43" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="48" t="inlineStr">
         <is>
           <t>สรุปการจัดกลุ่ม (ชุดเดียว) : กลุ่มหลัก → กลุ่มย่อย</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="45" t="inlineStr">
-        <is>
-          <t>กลุ่มหลักรวม 7 หมวดงาน + Software/Creative/Media/Marketing Metier (โครงการที่เป็นโอกาส Metier ยึดกลุ่ม Metier ก่อน · แถว Metier ไฮไลต์เหลือง)</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>กลุ่มย่อย Metier ใช้ canonical sub-service (Software/Creative/Media/Marketing)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>กลุ่มหลัก</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="48" t="inlineStr">
         <is>
           <t>กลุ่มย่อย</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="48" t="inlineStr">
         <is>
           <t>จำนวนโครงการ</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>ขอบเขต skill.md</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="37" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>1. บริหารจัดการ</t>
         </is>
       </c>
-      <c r="B5" s="37" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>บำรุงรักษา/ซ่อม</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
+      <c r="C5" t="n">
         <v>23</v>
       </c>
-      <c r="D5" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="37" t="n"/>
-      <c r="B6" s="37" t="inlineStr">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
         <is>
           <t>เช่า-จ้างเหมาบริการ (ทั่วไป)</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" t="n">
         <v>7</v>
       </c>
-      <c r="D6" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" s="37" t="n"/>
-      <c r="B7" s="37" t="inlineStr">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
         <is>
           <t>รักษาความปลอดภัย</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
     </row>
     <row r="8">
-      <c r="A8" s="37" t="n"/>
-      <c r="B8" s="37" t="inlineStr">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
         <is>
           <t>ระบบสารสนเทศ/ดิจิทัล/ซอฟต์แวร์</t>
         </is>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" s="37" t="n"/>
-      <c r="B9" s="37" t="inlineStr">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
         <is>
           <t>ป้องกันสาธารณภัย-ดับเพลิง</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
     </row>
     <row r="10">
-      <c r="A10" s="37" t="n"/>
-      <c r="B10" s="37" t="inlineStr">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
         <is>
           <t>เครือข่าย/อินเทอร์เน็ต/IT บริการ</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="37" t="n"/>
-      <c r="B11" s="37" t="inlineStr">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>จัดหาเครื่องแต่งกาย/วัสดุทั่วไป</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
         <is>
           <t>ฝึกอบรม-พัฒนาบุคลากร</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C12" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="37" t="n"/>
-      <c r="B12" s="37" t="inlineStr">
-        <is>
-          <t>จัดหาเครื่องแต่งกาย/วัสดุทั่วไป</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="n">
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>งานติดตั้ง/บริการอื่น</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ตรวจสอบ-ที่ปรึกษา</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>บริการสอบเทียบ/วิชาการ</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="48" t="inlineStr">
+        <is>
+          <t>รวม 1. บริหารจัดการ</t>
+        </is>
+      </c>
+      <c r="B16" s="48" t="inlineStr"/>
+      <c r="C16" s="48" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2. โครงสร้างพื้นฐาน</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>อาคาร/สิ่งก่อสร้าง/ลาน</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ประปา-แหล่งน้ำ</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ไฟฟ้า-แสงสว่าง/สาธารณูปโภค</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ถนน-คอนกรีต (คสล.)</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ถนน-แอสฟัลท์/ลาดยาง</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ถนน-บำรุง/ทั่วไป</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ระบบระบายน้ำ/ป้องกันตลิ่ง</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>งานระบบประกอบอาคาร (ปรับ/ระบายอากาศ)</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>วัสดุก่อสร้าง</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ไฟฟ้า-พลังงานแสงอาทิตย์</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>สะพาน/ทางเชื่อม</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="48" t="inlineStr">
+        <is>
+          <t>รวม 2. โครงสร้างพื้นฐาน</t>
+        </is>
+      </c>
+      <c r="B28" s="48" t="inlineStr"/>
+      <c r="C28" s="48" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>3. คุณภาพชีวิต</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>บริการตรวจวินิจฉัย/แล็บ</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>เวชภัณฑ์ยา/วัสดุการแพทย์</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>บริการสาธารณสุข</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>สวัสดิการ-ช่วยเหลือสังคม</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="48" t="inlineStr">
+        <is>
+          <t>รวม 3. คุณภาพชีวิต</t>
+        </is>
+      </c>
+      <c r="B33" s="48" t="inlineStr"/>
+      <c r="C33" s="48" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>4. ชุมชนเข้มแข็ง</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ชุมชน-ท่องเที่ยว-พลังงานชุมชน</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="48" t="inlineStr">
+        <is>
+          <t>รวม 4. ชุมชนเข้มแข็ง</t>
+        </is>
+      </c>
+      <c r="B35" s="48" t="inlineStr"/>
+      <c r="C35" s="48" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>5. การศึกษา ศาสนา กีฬา</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>สื่อ/อุปกรณ์การเรียนการสอน</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>สนามกีฬา</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="37" t="n"/>
-      <c r="B13" s="37" t="inlineStr">
-        <is>
-          <t>บริการสอบเทียบ/วิชาการ</t>
-        </is>
-      </c>
-      <c r="C13" s="14" t="n">
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>กีฬา-การแข่งขัน</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="37" t="n"/>
-      <c r="B14" s="37" t="inlineStr">
-        <is>
-          <t>งานติดตั้ง/บริการอื่น</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="n">
+    </row>
+    <row r="39">
+      <c r="A39" s="48" t="inlineStr">
+        <is>
+          <t>รวม 5. การศึกษา ศาสนา กีฬา</t>
+        </is>
+      </c>
+      <c r="B39" s="48" t="inlineStr"/>
+      <c r="C39" s="48" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>6. ความสะอาดและสิ่งแวดล้อม</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>กำจัดขยะ/ของเสีย</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ทำความสะอาด</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="48" t="inlineStr">
+        <is>
+          <t>รวม 6. ความสะอาดและสิ่งแวดล้อม</t>
+        </is>
+      </c>
+      <c r="B42" s="48" t="inlineStr"/>
+      <c r="C42" s="48" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>7. ครุภัณฑ์</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-วิทยาศาสตร์/การแพทย์</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-ยานพาหนะ</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์/วัสดุ-ดาราศาสตร์-วิจัย</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-คอมพิวเตอร์/IT</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-สำนักงาน</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-ก่อสร้าง/เครื่องจักร</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-โฆษณา/Display/CCTV</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์-ไฟฟ้าและวิทยุ</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="37" t="n"/>
-      <c r="B15" s="37" t="inlineStr">
-        <is>
-          <t>ตรวจสอบ-ที่ปรึกษา</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="n">
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ครุภัณฑ์/วัสดุ-โซลาร์</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>รวม 1. บริหารจัดการ</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="n"/>
-      <c r="C16" s="17" t="n">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="37" t="inlineStr">
-        <is>
-          <t>2. โครงสร้างพื้นฐาน</t>
-        </is>
-      </c>
-      <c r="B17" s="37" t="inlineStr">
-        <is>
-          <t>อาคาร/สิ่งก่อสร้าง/ลาน</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="n">
-        <v>21</v>
-      </c>
-      <c r="D17" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="37" t="n"/>
-      <c r="B18" s="37" t="inlineStr">
-        <is>
-          <t>ประปา-แหล่งน้ำ</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="D18" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="37" t="n"/>
-      <c r="B19" s="37" t="inlineStr">
-        <is>
-          <t>ไฟฟ้า-แสงสว่าง/สาธารณูปโภค</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="n">
-        <v>11</v>
-      </c>
-      <c r="D19" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="37" t="n"/>
-      <c r="B20" s="37" t="inlineStr">
-        <is>
-          <t>ถนน-คอนกรีต (คสล.)</t>
-        </is>
-      </c>
-      <c r="C20" s="14" t="n">
+    </row>
+    <row r="52">
+      <c r="A52" s="48" t="inlineStr">
+        <is>
+          <t>รวม 7. ครุภัณฑ์</t>
+        </is>
+      </c>
+      <c r="B52" s="48" t="inlineStr"/>
+      <c r="C52" s="48" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="49" t="inlineStr">
+        <is>
+          <t>Software Metier</t>
+        </is>
+      </c>
+      <c r="B53" s="49" t="inlineStr">
+        <is>
+          <t>ERP/CRM Systems</t>
+        </is>
+      </c>
+      <c r="C53" s="49" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="49" t="inlineStr"/>
+      <c r="B54" s="49" t="inlineStr">
+        <is>
+          <t>อื่น ๆ (ยังไม่จัดประเภท)</t>
+        </is>
+      </c>
+      <c r="C54" s="49" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="49" t="inlineStr"/>
+      <c r="B55" s="49" t="inlineStr">
+        <is>
+          <t>Mobile Application</t>
+        </is>
+      </c>
+      <c r="C55" s="49" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="49" t="inlineStr"/>
+      <c r="B56" s="49" t="inlineStr">
+        <is>
+          <t>Software Quality Assurance &amp; Cyber Security</t>
+        </is>
+      </c>
+      <c r="C56" s="49" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="48" t="inlineStr">
+        <is>
+          <t>รวม Software Metier</t>
+        </is>
+      </c>
+      <c r="B57" s="48" t="inlineStr"/>
+      <c r="C57" s="48" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="49" t="inlineStr">
+        <is>
+          <t>Creative Metier</t>
+        </is>
+      </c>
+      <c r="B58" s="49" t="inlineStr">
+        <is>
+          <t>Event Marketing</t>
+        </is>
+      </c>
+      <c r="C58" s="49" t="n">
         <v>10</v>
       </c>
-      <c r="D20" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="37" t="n"/>
-      <c r="B21" s="37" t="inlineStr">
-        <is>
-          <t>ถนน-แอสฟัลท์/ลาดยาง</t>
-        </is>
-      </c>
-      <c r="C21" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="D21" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="37" t="n"/>
-      <c r="B22" s="37" t="inlineStr">
-        <is>
-          <t>ระบบระบายน้ำ/ป้องกันตลิ่ง</t>
-        </is>
-      </c>
-      <c r="C22" s="14" t="n">
+    </row>
+    <row r="59">
+      <c r="A59" s="49" t="inlineStr"/>
+      <c r="B59" s="49" t="inlineStr">
+        <is>
+          <t>Content Creation</t>
+        </is>
+      </c>
+      <c r="C59" s="49" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="49" t="inlineStr"/>
+      <c r="B60" s="49" t="inlineStr">
+        <is>
+          <t>Graphic Design</t>
+        </is>
+      </c>
+      <c r="C60" s="49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="49" t="inlineStr"/>
+      <c r="B61" s="49" t="inlineStr">
+        <is>
+          <t>อื่น ๆ (ยังไม่จัดประเภท)</t>
+        </is>
+      </c>
+      <c r="C61" s="49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="48" t="inlineStr">
+        <is>
+          <t>รวม Creative Metier</t>
+        </is>
+      </c>
+      <c r="B62" s="48" t="inlineStr"/>
+      <c r="C62" s="48" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="49" t="inlineStr">
+        <is>
+          <t>Media Metier</t>
+        </is>
+      </c>
+      <c r="B63" s="49" t="inlineStr">
+        <is>
+          <t>Public Relations</t>
+        </is>
+      </c>
+      <c r="C63" s="49" t="n">
         <v>4</v>
       </c>
-      <c r="D22" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="37" t="n"/>
-      <c r="B23" s="37" t="inlineStr">
-        <is>
-          <t>ถนน-บำรุง/ทั่วไป</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D23" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="37" t="n"/>
-      <c r="B24" s="37" t="inlineStr">
-        <is>
-          <t>วัสดุก่อสร้าง</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="D24" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="37" t="n"/>
-      <c r="B25" s="37" t="inlineStr">
-        <is>
-          <t>งานระบบประกอบอาคาร (ปรับ/ระบายอากาศ)</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="D25" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="37" t="n"/>
-      <c r="B26" s="37" t="inlineStr">
-        <is>
-          <t>ไฟฟ้า-พลังงานแสงอาทิตย์</t>
-        </is>
-      </c>
-      <c r="C26" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="D26" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="37" t="n"/>
-      <c r="B27" s="37" t="inlineStr">
-        <is>
-          <t>สะพาน/ทางเชื่อม</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="n">
+    </row>
+    <row r="64">
+      <c r="A64" s="49" t="inlineStr"/>
+      <c r="B64" s="49" t="inlineStr">
+        <is>
+          <t>Offline Media</t>
+        </is>
+      </c>
+      <c r="C64" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="D27" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>รวม 2. โครงสร้างพื้นฐาน</t>
-        </is>
-      </c>
-      <c r="B28" s="16" t="n"/>
-      <c r="C28" s="17" t="n">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="37" t="inlineStr">
-        <is>
-          <t>3. คุณภาพชีวิต</t>
-        </is>
-      </c>
-      <c r="B29" s="37" t="inlineStr">
-        <is>
-          <t>บริการตรวจวินิจฉัย/แล็บ</t>
-        </is>
-      </c>
-      <c r="C29" s="14" t="n">
-        <v>16</v>
-      </c>
-      <c r="D29" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="37" t="n"/>
-      <c r="B30" s="37" t="inlineStr">
-        <is>
-          <t>เวชภัณฑ์ยา/วัสดุการแพทย์</t>
-        </is>
-      </c>
-      <c r="C30" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="D30" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="37" t="n"/>
-      <c r="B31" s="37" t="inlineStr">
-        <is>
-          <t>บริการสาธารณสุข</t>
-        </is>
-      </c>
-      <c r="C31" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="D31" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="37" t="n"/>
-      <c r="B32" s="37" t="inlineStr">
-        <is>
-          <t>สวัสดิการ-ช่วยเหลือสังคม</t>
-        </is>
-      </c>
-      <c r="C32" s="14" t="n">
+    </row>
+    <row r="65">
+      <c r="A65" s="48" t="inlineStr">
+        <is>
+          <t>รวม Media Metier</t>
+        </is>
+      </c>
+      <c r="B65" s="48" t="inlineStr"/>
+      <c r="C65" s="48" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="49" t="inlineStr">
+        <is>
+          <t>Marketing Metier</t>
+        </is>
+      </c>
+      <c r="B66" s="49" t="inlineStr">
+        <is>
+          <t>Brand Strategy</t>
+        </is>
+      </c>
+      <c r="C66" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="D32" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
-        <is>
-          <t>รวม 3. คุณภาพชีวิต</t>
-        </is>
-      </c>
-      <c r="B33" s="16" t="n"/>
-      <c r="C33" s="17" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="37" t="inlineStr">
-        <is>
-          <t>4. ชุมชนเข้มแข็ง</t>
-        </is>
-      </c>
-      <c r="B34" s="37" t="inlineStr">
-        <is>
-          <t>ชุมชน-ท่องเที่ยว-พลังงานชุมชน</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D34" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="15" t="inlineStr">
-        <is>
-          <t>รวม 4. ชุมชนเข้มแข็ง</t>
-        </is>
-      </c>
-      <c r="B35" s="16" t="n"/>
-      <c r="C35" s="17" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="37" t="inlineStr">
-        <is>
-          <t>5. การศึกษา ศาสนา กีฬา</t>
-        </is>
-      </c>
-      <c r="B36" s="37" t="inlineStr">
-        <is>
-          <t>สื่อ/อุปกรณ์การเรียนการสอน</t>
-        </is>
-      </c>
-      <c r="C36" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D36" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="37" t="n"/>
-      <c r="B37" s="37" t="inlineStr">
-        <is>
-          <t>สนามกีฬา</t>
-        </is>
-      </c>
-      <c r="C37" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D37" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="37" t="n"/>
-      <c r="B38" s="37" t="inlineStr">
-        <is>
-          <t>กีฬา-การแข่งขัน</t>
-        </is>
-      </c>
-      <c r="C38" s="14" t="n">
+    </row>
+    <row r="67">
+      <c r="A67" s="48" t="inlineStr">
+        <is>
+          <t>รวม Marketing Metier</t>
+        </is>
+      </c>
+      <c r="B67" s="48" t="inlineStr"/>
+      <c r="C67" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="D38" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="15" t="inlineStr">
-        <is>
-          <t>รวม 5. การศึกษา ศาสนา กีฬา</t>
-        </is>
-      </c>
-      <c r="B39" s="16" t="n"/>
-      <c r="C39" s="17" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="37" t="inlineStr">
-        <is>
-          <t>6. ความสะอาดและสิ่งแวดล้อม</t>
-        </is>
-      </c>
-      <c r="B40" s="37" t="inlineStr">
-        <is>
-          <t>กำจัดขยะ/ของเสีย</t>
-        </is>
-      </c>
-      <c r="C40" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="D40" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="37" t="n"/>
-      <c r="B41" s="37" t="inlineStr">
-        <is>
-          <t>ทำความสะอาด</t>
-        </is>
-      </c>
-      <c r="C41" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="D41" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="15" t="inlineStr">
-        <is>
-          <t>รวม 6. ความสะอาดและสิ่งแวดล้อม</t>
-        </is>
-      </c>
-      <c r="B42" s="16" t="n"/>
-      <c r="C42" s="17" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="37" t="inlineStr">
-        <is>
-          <t>7. ครุภัณฑ์</t>
-        </is>
-      </c>
-      <c r="B43" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-วิทยาศาสตร์/การแพทย์</t>
-        </is>
-      </c>
-      <c r="C43" s="14" t="n">
-        <v>20</v>
-      </c>
-      <c r="D43" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="37" t="n"/>
-      <c r="B44" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-ยานพาหนะ</t>
-        </is>
-      </c>
-      <c r="C44" s="14" t="n">
-        <v>18</v>
-      </c>
-      <c r="D44" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="37" t="n"/>
-      <c r="B45" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์/วัสดุ-ดาราศาสตร์-วิจัย</t>
-        </is>
-      </c>
-      <c r="C45" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="D45" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="37" t="n"/>
-      <c r="B46" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-คอมพิวเตอร์/IT</t>
-        </is>
-      </c>
-      <c r="C46" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="D46" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="37" t="n"/>
-      <c r="B47" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-สำนักงาน</t>
-        </is>
-      </c>
-      <c r="C47" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D47" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="37" t="n"/>
-      <c r="B48" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-ก่อสร้าง/เครื่องจักร</t>
-        </is>
-      </c>
-      <c r="C48" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D48" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="37" t="n"/>
-      <c r="B49" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-โฆษณา/Display/CCTV</t>
-        </is>
-      </c>
-      <c r="C49" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D49" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="37" t="n"/>
-      <c r="B50" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์-ไฟฟ้าและวิทยุ</t>
-        </is>
-      </c>
-      <c r="C50" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="37" t="n"/>
-      <c r="B51" s="37" t="inlineStr">
-        <is>
-          <t>ครุภัณฑ์/วัสดุ-โซลาร์</t>
-        </is>
-      </c>
-      <c r="C51" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" s="37" t="inlineStr">
-        <is>
-          <t>ภาพรวม (stub)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="15" t="inlineStr">
-        <is>
-          <t>รวม 7. ครุภัณฑ์</t>
-        </is>
-      </c>
-      <c r="B52" s="16" t="n"/>
-      <c r="C52" s="17" t="n">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="26" t="inlineStr">
-        <is>
-          <t>Software Metier</t>
-        </is>
-      </c>
-      <c r="B53" s="37" t="inlineStr">
-        <is>
-          <t>System Development</t>
-        </is>
-      </c>
-      <c r="C53" s="14" t="n">
-        <v>19</v>
-      </c>
-      <c r="D53" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="37" t="n"/>
-      <c r="B54" s="37" t="inlineStr">
-        <is>
-          <t>Smart City/Platform Development</t>
-        </is>
-      </c>
-      <c r="C54" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D54" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="37" t="n"/>
-      <c r="B55" s="37" t="inlineStr">
-        <is>
-          <t>Cybersecurity/Certificate</t>
-        </is>
-      </c>
-      <c r="C55" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="D55" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="37" t="n"/>
-      <c r="B56" s="37" t="inlineStr">
-        <is>
-          <t>Software/License</t>
-        </is>
-      </c>
-      <c r="C56" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="37" t="n"/>
-      <c r="B57" s="37" t="inlineStr">
-        <is>
-          <t>Mobile Application</t>
-        </is>
-      </c>
-      <c r="C57" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D57" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="27" t="inlineStr">
-        <is>
-          <t>รวม Software Metier</t>
-        </is>
-      </c>
-      <c r="B58" s="28" t="n"/>
-      <c r="C58" s="29" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="26" t="inlineStr">
-        <is>
-          <t>Creative Metier</t>
-        </is>
-      </c>
-      <c r="B59" s="37" t="inlineStr">
-        <is>
-          <t>Event Marketing/Festival</t>
-        </is>
-      </c>
-      <c r="C59" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="D59" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="37" t="n"/>
-      <c r="B60" s="37" t="inlineStr">
-        <is>
-          <t>Content Creation / Graphic Design</t>
-        </is>
-      </c>
-      <c r="C60" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D60" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="37" t="n"/>
-      <c r="B61" s="37" t="inlineStr">
-        <is>
-          <t>Branding &amp; Display Production</t>
-        </is>
-      </c>
-      <c r="C61" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="27" t="inlineStr">
-        <is>
-          <t>รวม Creative Metier</t>
-        </is>
-      </c>
-      <c r="B62" s="28" t="n"/>
-      <c r="C62" s="29" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="26" t="inlineStr">
-        <is>
-          <t>Media Metier</t>
-        </is>
-      </c>
-      <c r="B63" s="37" t="inlineStr">
-        <is>
-          <t>Public Relations</t>
-        </is>
-      </c>
-      <c r="C63" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D63" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="37" t="n"/>
-      <c r="B64" s="37" t="inlineStr">
-        <is>
-          <t>Offline Media</t>
-        </is>
-      </c>
-      <c r="C64" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="27" t="inlineStr">
-        <is>
-          <t>รวม Media Metier</t>
-        </is>
-      </c>
-      <c r="B65" s="28" t="n"/>
-      <c r="C65" s="29" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="26" t="inlineStr">
-        <is>
-          <t>Marketing Metier</t>
-        </is>
-      </c>
-      <c r="B66" s="37" t="inlineStr">
-        <is>
-          <t>Brand/Corporate Image</t>
-        </is>
-      </c>
-      <c r="C66" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="37" t="inlineStr">
-        <is>
-          <t>⭐ มีรายละเอียดกลุ่มย่อย (skill 08–11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="27" t="inlineStr">
-        <is>
-          <t>รวม Marketing Metier</t>
-        </is>
-      </c>
-      <c r="B67" s="28" t="n"/>
-      <c r="C67" s="29" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="68">
-      <c r="A68" s="18" t="inlineStr">
+      <c r="A68" s="48" t="inlineStr">
         <is>
           <t>รวมทั้งหมด</t>
         </is>
       </c>
-      <c r="B68" s="18" t="n"/>
-      <c r="C68" s="1" t="n">
+      <c r="B68" s="48" t="inlineStr"/>
+      <c r="C68" s="48" t="n">
         <v>310</v>
       </c>
     </row>
-    <row r="69"/>
-    <row r="70">
-      <c r="A70" s="44" t="inlineStr">
-        <is>
-          <t>➜ โครงการที่เป็นโอกาส Metier (Software/Creative/Media/Marketing Metier) = 49 จาก 310 โครงการ</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A70:C70"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>